<commit_message>
Add per-run provenance and GPU validation evidence
</commit_message>
<xml_diff>
--- a/submissions/2A202602982_HaManhTuan/results.xlsx
+++ b/submissions/2A202602982_HaManhTuan/results.xlsx
@@ -14,15 +14,17 @@
     <sheet name="PerClass" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Latency" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="BackboneLatency" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backbones'!$A$1:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backbones'!$A$1:$N$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$M$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$K$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Final'!$A$1:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PerClass'!$A$1:$G$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Latency'!$A$1:$N$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Summary'!$A$1:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'BackboneLatency'!$A$1:$N$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,16 +33,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -51,7 +50,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -59,21 +58,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,63 +429,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>backbone</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pretrained_tag</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>params_m</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>best_epoch</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>macro_f1_val</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>top1_val</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ece_val</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>seconds_per_epoch</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>gmac</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>latency_p50_ms</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>latency_p95_ms</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>latency_p99_ms</t>
         </is>
       </c>
     </row>
@@ -539,6 +544,15 @@
       <c r="K2" t="n">
         <v>4.109483008</v>
       </c>
+      <c r="L2" t="n">
+        <v>5.611932137981057</v>
+      </c>
+      <c r="M2" t="n">
+        <v>5.64943163190037</v>
+      </c>
+      <c r="N2" t="n">
+        <v>5.658592879772186</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -580,6 +594,15 @@
       <c r="K3" t="n">
         <v>1.818558464</v>
       </c>
+      <c r="L3" t="n">
+        <v>2.317859558388591</v>
+      </c>
+      <c r="M3" t="n">
+        <v>2.353760856203735</v>
+      </c>
+      <c r="N3" t="n">
+        <v>2.386640105396509</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -621,6 +644,15 @@
       <c r="K4" t="n">
         <v>3.670755328</v>
       </c>
+      <c r="L4" t="n">
+        <v>4.163214936852455</v>
+      </c>
+      <c r="M4" t="n">
+        <v>4.196777334436774</v>
+      </c>
+      <c r="N4" t="n">
+        <v>4.203253984451294</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -662,6 +694,15 @@
       <c r="K5" t="n">
         <v>0.203019328</v>
       </c>
+      <c r="L5" t="n">
+        <v>4.803354619070888</v>
+      </c>
+      <c r="M5" t="n">
+        <v>4.867686820216477</v>
+      </c>
+      <c r="N5" t="n">
+        <v>4.877639166079462</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -703,6 +744,15 @@
       <c r="K6" t="n">
         <v>1.079389056</v>
       </c>
+      <c r="L6" t="n">
+        <v>4.20006038621068</v>
+      </c>
+      <c r="M6" t="n">
+        <v>4.230727371759713</v>
+      </c>
+      <c r="N6" t="n">
+        <v>4.996608505025504</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -744,9 +794,18 @@
       <c r="K7" t="n">
         <v>4.25735168</v>
       </c>
+      <c r="L7" t="n">
+        <v>5.572114838287234</v>
+      </c>
+      <c r="M7" t="n">
+        <v>5.623853020370007</v>
+      </c>
+      <c r="N7" t="n">
+        <v>5.665736813098192</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K7"/>
+  <autoFilter ref="A1:N7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -761,67 +820,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>backbone</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pretrained_tag</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>params_m</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>best_epoch</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>macro_f1_val</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>top1_val</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ece_val</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>seconds_per_epoch</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>gmac</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>axis</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>change</t>
         </is>
@@ -1192,57 +1251,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>macro_f1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>top1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>balanced_acc</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ece</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>nll</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>latency_p50_ms</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>latency_p95_ms</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>latency_p99_ms</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>relative_cost</t>
         </is>
@@ -1819,42 +1878,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>macro_f1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>top1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>balanced_acc</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ece</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>nll</t>
         </is>
@@ -2056,37 +2115,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>f1</t>
         </is>
@@ -3566,72 +3625,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>p50</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>p95</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>p99</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>mean</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>gpu</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>dtype</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>batch</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>img_size</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>images_per_s</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>torch</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>preprocessing_included</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>k_views</t>
         </is>
@@ -3885,67 +3944,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>backbone</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pretrained_tag</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>params_m</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>best_epoch</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>macro_f1_val</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>top1_val</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ece_val</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>seconds_per_epoch</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>gmac</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>axis</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>change</t>
         </is>
@@ -4417,4 +4476,415 @@
   <autoFilter ref="A1:M11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>exp_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>backbone</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>p50</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>p99</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>gpu</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dtype</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>img_size</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>images_per_s</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>torch</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>preprocessing_included</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5.611932137981057</v>
+      </c>
+      <c r="D2" t="n">
+        <v>5.64943163190037</v>
+      </c>
+      <c r="E2" t="n">
+        <v>5.658592879772186</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5.605953801423311</v>
+      </c>
+      <c r="G2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3090</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>224</v>
+      </c>
+      <c r="L2" t="n">
+        <v>178.1917484768016</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2.6.0+cu124</t>
+        </is>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>resnet18</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2.317859558388591</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.353760856203735</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.386640105396509</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.319932552054524</v>
+      </c>
+      <c r="G3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3090</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>224</v>
+      </c>
+      <c r="L3" t="n">
+        <v>431.4325241928007</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2.6.0+cu124</t>
+        </is>
+      </c>
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>resnet34</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>4.163214936852455</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4.196777334436774</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4.203253984451294</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.164046039804816</v>
+      </c>
+      <c r="G4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3090</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>224</v>
+      </c>
+      <c r="L4" t="n">
+        <v>240.1989844790567</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2.6.0+cu124</t>
+        </is>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>regnetx_002</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4.803354619070888</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4.867686820216477</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4.877639166079462</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.809023132547736</v>
+      </c>
+      <c r="G5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3090</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>224</v>
+      </c>
+      <c r="L5" t="n">
+        <v>208.1878352328336</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2.6.0+cu124</t>
+        </is>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4.20006038621068</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4.230727371759713</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.996608505025504</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.232073873281479</v>
+      </c>
+      <c r="G6" t="n">
+        <v>50</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3090</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>224</v>
+      </c>
+      <c r="L6" t="n">
+        <v>238.0918148898821</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2.6.0+cu124</t>
+        </is>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>resnext50_32x4d</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5.572114838287234</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5.623853020370007</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5.665736813098192</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5.572382267564535</v>
+      </c>
+      <c r="G7" t="n">
+        <v>50</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3090</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>224</v>
+      </c>
+      <c r="L7" t="n">
+        <v>179.4650736788084</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2.6.0+cu124</t>
+        </is>
+      </c>
+      <c r="N7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Finalize DeepWeeds submission against rubric
</commit_message>
<xml_diff>
--- a/submissions/2A202602982_HaManhTuan/results.xlsx
+++ b/submissions/2A202602982_HaManhTuan/results.xlsx
@@ -17,13 +17,13 @@
     <sheet name="BackboneLatency" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backbones'!$A$1:$N$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$M$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$K$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Final'!$A$1:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backbones'!$A$1:$Q$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training'!$A$1:$Q$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$P$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Final'!$A$1:$R$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PerClass'!$A$1:$G$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Latency'!$A$1:$N$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Summary'!$A$1:$M$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Latency'!$A$1:$P$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Summary'!$A$1:$O$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'BackboneLatency'!$A$1:$N$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,13 +41,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017365D"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -62,8 +71,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,78 +439,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="17" max="17"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>backbone</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pretrained_tag</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>params_m</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>best_epoch</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>macro_f1_val</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>top1_val</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ece_val</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>seconds_per_epoch</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>gmac</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>latency_p50_ms</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>latency_p95_ms</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>latency_p99_ms</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>img_size_px</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>epochs</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
@@ -553,6 +597,17 @@
       <c r="N2" t="n">
         <v>5.658592879772186</v>
       </c>
+      <c r="O2" t="n">
+        <v>224</v>
+      </c>
+      <c r="P2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>original screening</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -603,6 +658,17 @@
       <c r="N3" t="n">
         <v>2.386640105396509</v>
       </c>
+      <c r="O3" t="n">
+        <v>224</v>
+      </c>
+      <c r="P3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>original screening</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -653,6 +719,17 @@
       <c r="N4" t="n">
         <v>4.203253984451294</v>
       </c>
+      <c r="O4" t="n">
+        <v>224</v>
+      </c>
+      <c r="P4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>original screening</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -703,6 +780,17 @@
       <c r="N5" t="n">
         <v>4.877639166079462</v>
       </c>
+      <c r="O5" t="n">
+        <v>224</v>
+      </c>
+      <c r="P5" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>original screening</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -753,6 +841,17 @@
       <c r="N6" t="n">
         <v>4.996608505025504</v>
       </c>
+      <c r="O6" t="n">
+        <v>224</v>
+      </c>
+      <c r="P6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>original screening</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -803,9 +902,20 @@
       <c r="N7" t="n">
         <v>5.665736813098192</v>
       </c>
+      <c r="O7" t="n">
+        <v>224</v>
+      </c>
+      <c r="P7" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>supplemented after final selection</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N7"/>
+  <autoFilter ref="A1:Q7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -816,73 +926,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="29" customWidth="1" min="17" max="17"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>backbone</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pretrained_tag</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>params_m</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>best_epoch</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>macro_f1_val</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>top1_val</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ece_val</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>seconds_per_epoch</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>gmac</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>axis</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>change</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>delta_macro_f1_vs_T00</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>chinee_apple_f1_val</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>snake_weed_f1_val</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
@@ -928,6 +1077,20 @@
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.8317307692307692</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.8706467661691542</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -979,6 +1142,20 @@
           <t>{"init": "frozen"}</t>
         </is>
       </c>
+      <c r="N3" t="n">
+        <v>-0.3241052975457404</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.5288461538461539</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.5646437994722955</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>one factor changed from T00</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1030,6 +1207,20 @@
           <t>{"init": "scratch"}</t>
         </is>
       </c>
+      <c r="N4" t="n">
+        <v>-0.3149530049011532</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.4881516587677726</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.4717607973421927</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>one factor changed from T00</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1081,6 +1272,20 @@
           <t>{"aug": "color"}</t>
         </is>
       </c>
+      <c r="N5" t="n">
+        <v>0.001483242823741904</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.8551068883610451</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.8693467336683417</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>one factor changed from T00</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1132,6 +1337,20 @@
           <t>{"aug": "randaug"}</t>
         </is>
       </c>
+      <c r="N6" t="n">
+        <v>0.007002114341856158</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.8516746411483253</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.882051282051282</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>one factor changed from T00</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1183,6 +1402,20 @@
           <t>{"loss": "ls", "label_smoothing": 0.1}</t>
         </is>
       </c>
+      <c r="N7" t="n">
+        <v>-0.009598502610338011</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.8280871670702179</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.8557213930348258</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>one factor changed from T00</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1234,9 +1467,23 @@
           <t>{"loss": "focal", "focal_gamma": 2.0}</t>
         </is>
       </c>
+      <c r="N8" t="n">
+        <v>-0.01895498136915275</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.8094117647058824</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.846938775510204</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>one factor changed from T00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M8"/>
+  <autoFilter ref="A1:Q8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1247,63 +1494,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>macro_f1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>top1</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>balanced_acc</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ece</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>nll</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>latency_p50_ms</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>latency_p95_ms</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>latency_p99_ms</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>relative_cost</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>method_description</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>views</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>backbone</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>checkpoint</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>images_per_s_batch1</t>
         </is>
       </c>
     </row>
@@ -1343,6 +1633,27 @@
       <c r="K2" t="n">
         <v>1</v>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>one view</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>F01_seed0</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>222.4577378097799</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1380,6 +1691,27 @@
       <c r="K3" t="n">
         <v>1.901401473701799</v>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>horizontal flip; mean probabilities</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>F01_seed0</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>116.9967210431796</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1417,6 +1749,27 @@
       <c r="K4" t="n">
         <v>1.901401473701799</v>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>horizontal flip; mean logits</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>F01_seed0</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>116.9967210431796</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1454,6 +1807,27 @@
       <c r="K5" t="n">
         <v>1</v>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>one view; temperature scaling</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>F01_seed0</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>222.4577378097799</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1491,6 +1865,27 @@
       <c r="K6" t="n">
         <v>1.901401473701799</v>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>horizontal flip; mean logits; temperature scaling</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>F01_seed0</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>116.9967210431796</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1528,6 +1923,27 @@
       <c r="K7" t="n">
         <v>1</v>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>one view</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>F01_seed1</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>222.4577378097799</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1565,6 +1981,27 @@
       <c r="K8" t="n">
         <v>1.901401473701799</v>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>horizontal flip; mean probabilities</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>F01_seed1</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>116.9967210431796</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1602,6 +2039,27 @@
       <c r="K9" t="n">
         <v>1.901401473701799</v>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>horizontal flip; mean logits</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>F01_seed1</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>116.9967210431796</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1639,6 +2097,27 @@
       <c r="K10" t="n">
         <v>1</v>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>one view; temperature scaling</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>F01_seed1</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>222.4577378097799</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1676,6 +2155,27 @@
       <c r="K11" t="n">
         <v>1.901401473701799</v>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>horizontal flip; mean logits; temperature scaling</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>F01_seed1</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>116.9967210431796</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1713,6 +2213,27 @@
       <c r="K12" t="n">
         <v>1</v>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>one view</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>F01_seed2</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>222.4577378097799</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1750,6 +2271,27 @@
       <c r="K13" t="n">
         <v>1.901401473701799</v>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>horizontal flip; mean probabilities</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>F01_seed2</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>116.9967210431796</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1787,6 +2329,27 @@
       <c r="K14" t="n">
         <v>1.901401473701799</v>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>horizontal flip; mean logits</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>F01_seed2</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>116.9967210431796</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1824,6 +2387,27 @@
       <c r="K15" t="n">
         <v>1</v>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>one view; temperature scaling</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>F01_seed2</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>222.4577378097799</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1861,9 +2445,30 @@
       <c r="K16" t="n">
         <v>1.901401473701799</v>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>horizontal flip; mean logits; temperature scaling</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>F01_seed2</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>116.9967210431796</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K16"/>
+  <autoFilter ref="A1:P16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1874,48 +2479,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>macro_f1</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>top1</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>balanced_acc</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ece</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>nll</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>backbone</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1_test_mean</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1_test_std</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>top1_test_mean</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>top1_test_std</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>ece_test_mean</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>ece_test_std</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>macro_f1_val</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>top1_val</t>
         </is>
       </c>
     </row>
@@ -1948,6 +2623,40 @@
       <c r="H2" t="n">
         <v>0.1988500115723452</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>basic augmentation; CE</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.9187108509311323</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.006052743892057421</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.9392643284858854</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.004588958351705446</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.01907954653526201</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.005020100801482854</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.918270992883581</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.9385889745786918</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1978,6 +2687,40 @@
       <c r="H3" t="n">
         <v>0.189941892275061</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>basic augmentation; CE</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.9187108509311323</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.006052743892057421</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.9392643284858854</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.004588958351705446</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.01907954653526201</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.005020100801482854</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.9256573564786323</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.9445872607826336</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2008,6 +2751,40 @@
       <c r="H4" t="n">
         <v>0.1820005618709453</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>basic augmentation; CE</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.9187108509311323</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.006052743892057421</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.9392643284858854</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.004588958351705446</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.01907954653526201</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.005020100801482854</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.9206273664819835</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.9414453013424736</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2038,6 +2815,40 @@
       <c r="H5" t="n">
         <v>0.1529435217380524</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>RandAugment; CE</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.9327133106514539</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.002854264704167327</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.9483889364128886</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.003084303913998267</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.01211940454174478</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.001829236136130228</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.932312400404177</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.9491573836046844</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2068,6 +2879,40 @@
       <c r="H6" t="n">
         <v>0.1522357314825058</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>RandAugment; CE</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.9327133106514539</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.002854264704167327</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.9483889364128886</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.003084303913998267</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.01211940454174478</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.001829236136130228</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.9308786645845597</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.9465866895172808</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2098,9 +2943,43 @@
       <c r="H7" t="n">
         <v>0.1603932827711105</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>vit_tiny_patch16_224</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>RandAugment; CE</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0.9327133106514539</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.002854264704167327</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.9483889364128886</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.003084303913998267</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.01211940454174478</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.001829236136130228</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.9317652478095577</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.9468723221936589</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
+  <autoFilter ref="A1:R7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2113,39 +2992,48 @@
   </sheetPr>
   <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>class</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>support</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precision</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>recall</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>f1</t>
         </is>
@@ -3621,78 +4509,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>p50</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>p95</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>p99</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>mean</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>gpu</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>dtype</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>batch</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>img_size</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>images_per_s</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>torch</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>preprocessing_included</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>k_views</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>configuration</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>bn_fused</t>
         </is>
       </c>
     </row>
@@ -3745,6 +4661,14 @@
         <v>0</v>
       </c>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>ViT Tiny; I00</t>
+        </is>
+      </c>
+      <c r="P2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3795,6 +4719,14 @@
         <v>0</v>
       </c>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>ViT Tiny; I00</t>
+        </is>
+      </c>
+      <c r="P3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3845,6 +4777,14 @@
         <v>0</v>
       </c>
       <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>ViT Tiny; I00</t>
+        </is>
+      </c>
+      <c r="P4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3895,6 +4835,14 @@
         <v>0</v>
       </c>
       <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>ViT Tiny; I00</t>
+        </is>
+      </c>
+      <c r="P5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3917,19 +4865,39 @@
       <c r="F6" t="n">
         <v>50</v>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>NVIDIA GeForce RTX 3090</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>116.9967210431796</v>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
         <v>2</v>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>ViT Tiny; I01/I02/I04</t>
+        </is>
+      </c>
+      <c r="P6" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N6"/>
+  <autoFilter ref="A1:P6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3940,73 +4908,100 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>backbone</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pretrained_tag</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>params_m</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>best_epoch</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>macro_f1_val</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>top1_val</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ece_val</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>seconds_per_epoch</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>gmac</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>axis</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>change</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>latency_p95_ms</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>rank_val_macro_f1</t>
         </is>
       </c>
     </row>
@@ -4060,6 +5055,12 @@
           <t>{"aug": "randaug"}</t>
         </is>
       </c>
+      <c r="N2" t="n">
+        <v>4.230727371759713</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4111,6 +5112,12 @@
           <t>{"aug": "color"}</t>
         </is>
       </c>
+      <c r="N3" t="n">
+        <v>4.230727371759713</v>
+      </c>
+      <c r="O3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4154,6 +5161,12 @@
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="n">
+        <v>4.230727371759713</v>
+      </c>
+      <c r="O4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4197,6 +5210,12 @@
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="n">
+        <v>4.230727371759713</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4248,6 +5267,12 @@
           <t>{"loss": "ls", "label_smoothing": 0.1}</t>
         </is>
       </c>
+      <c r="N6" t="n">
+        <v>4.230727371759713</v>
+      </c>
+      <c r="O6" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4299,6 +5324,12 @@
           <t>{"loss": "focal", "focal_gamma": 2.0}</t>
         </is>
       </c>
+      <c r="N7" t="n">
+        <v>4.230727371759713</v>
+      </c>
+      <c r="O7" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4342,6 +5373,12 @@
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
+      <c r="N8" t="n">
+        <v>4.867686820216477</v>
+      </c>
+      <c r="O8" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4385,6 +5422,12 @@
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
+      <c r="N9" t="n">
+        <v>5.64943163190037</v>
+      </c>
+      <c r="O9" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4428,6 +5471,12 @@
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>5.623853020370007</v>
+      </c>
+      <c r="O10" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4471,9 +5520,15 @@
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>2.353760856203735</v>
+      </c>
+      <c r="O11" t="n">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M11"/>
+  <autoFilter ref="A1:O11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4486,74 +5541,90 @@
   </sheetPr>
   <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>exp_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>backbone</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>p50</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>p95</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>p99</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>mean</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>gpu</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>dtype</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>batch</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>img_size</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>images_per_s</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>torch</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>preprocessing_included</t>
         </is>

</xml_diff>